<commit_message>
Localize the shop for Taiwan and sync TWD prices from the product list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/product_list.xlsx
+++ b/product_list.xlsx
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10">
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12">
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15">
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16">
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17">
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19">
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20">
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21">
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22">
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23">
@@ -1184,7 +1184,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28">
@@ -1334,7 +1334,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37">
@@ -1604,7 +1604,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="38">
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39">
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="40">
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41">
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="42">
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43">
@@ -1784,7 +1784,7 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="44">
@@ -1814,7 +1814,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45">
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="46">
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47">
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="48">
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49">
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="50">
@@ -1994,7 +1994,7 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="51">
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="52">
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="53">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="54">
@@ -2114,7 +2114,7 @@
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55">
@@ -2144,7 +2144,7 @@
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="56">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57">
@@ -2204,7 +2204,7 @@
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="58">
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59">
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="60">
@@ -2294,7 +2294,7 @@
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="61">
@@ -2324,7 +2324,7 @@
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="62">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63">
@@ -2384,7 +2384,7 @@
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="64">
@@ -2414,7 +2414,7 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="65">
@@ -2444,7 +2444,7 @@
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="66">
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="67">
@@ -2504,7 +2504,7 @@
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="68">
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="69">
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="70">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="71">
@@ -2624,7 +2624,7 @@
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="72">
@@ -2654,7 +2654,7 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="73">
@@ -2684,7 +2684,7 @@
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="74">
@@ -2714,7 +2714,7 @@
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="75">
@@ -2744,7 +2744,7 @@
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="76">
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77">
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="78">
@@ -2834,7 +2834,7 @@
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="79">
@@ -2864,7 +2864,7 @@
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="80">
@@ -2894,7 +2894,7 @@
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="81">
@@ -2924,7 +2924,7 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="82">
@@ -2954,7 +2954,7 @@
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="83">
@@ -2984,7 +2984,7 @@
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="84">
@@ -3014,7 +3014,7 @@
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="85">
@@ -3044,7 +3044,7 @@
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="86">
@@ -3074,7 +3074,7 @@
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="87">
@@ -3104,7 +3104,7 @@
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="88">
@@ -3134,7 +3134,7 @@
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="89">
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="90">
@@ -3194,7 +3194,7 @@
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="91">
@@ -3224,7 +3224,7 @@
         </is>
       </c>
       <c r="F91" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="92">
@@ -3254,7 +3254,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="93">
@@ -3284,7 +3284,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="94">
@@ -3314,7 +3314,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="95">
@@ -3344,7 +3344,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="96">
@@ -3374,7 +3374,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="97">
@@ -3404,7 +3404,7 @@
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
     </row>
     <row r="98">

</xml_diff>